<commit_message>
feat: typing/terminal SFX pack + terminal_flow BGM, sync docs & branding
</commit_message>
<xml_diff>
--- a/guides/audio-library.xlsx
+++ b/guides/audio-library.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="چک‌لیست نهایی" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'افکت‌های صوتی'!$A$1:$G$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'موسیقی پس‌زمینه'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'افکت‌های صوتی'!$A$1:$G$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'موسیقی پس‌زمینه'!$A$1:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'منابع رایگان'!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'کلمات کلیدی جستجو'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'الگوی تایم‌لاین'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'الگوی تایم‌لاین'!$A$1:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'تنظیم سطح صدا'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'چک‌لیست نهایی'!$A$1:$B$13</definedName>
   </definedNames>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1596,79 +1596,412 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>فضاسازی (لوپ)</t>
+          <t>تایپ و ترمینال</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>room_tone_loop</t>
+          <t>type_key_single</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>نویز اتاق + هوم + فن</t>
+          <t>تک‌کلید مکانیکی</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>زیر کل ویدیو برای پرکردن سکوت مطلق</t>
+          <t>همگام‌سازی با کلیدهای دیده‌شده روی تصویر</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Loop از ابتدا تا انتها، بدون قطع</t>
+          <t>روی فریم فشردن کلید</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>−۳۴ تا −۳۰ dB</t>
+          <t>−۱۲ dB</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>30.00s</t>
+          <t>0.05s</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>type_burst_mech</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>تایپ مکانیکی کلیکی</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>تایپ کد وقتی روی تصویر دیده می‌شود</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>با Rate Stretch همگام کن</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>−۱۶ dB</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2.80s</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>type_burst_soft</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>تایپ نرم</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>تایپ زیر نریشن، جلسه‌های طولانی</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Loop یا زنجیره‌ای</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>−۱۸ dB</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>3.20s</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>type_key_roll</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>رگبار ۷ کلید</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>تایپ سریع دستور بلند</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>روی شروع تایپ دستور</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>−۱۳ dB</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>0.50s</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>type_enter</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>کلید Enter</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>لحظه‌ی اجرای دستور در ترمینال</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>دقیقاً روی فریم Enter</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>−۱۰ dB</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>0.10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>type_backspace</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>کلید Backspace</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>حذف/اصلاح</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>روی فریم حذف</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>−۱۲ dB</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>0.05s</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>terminal_bell</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>زنگ کلاسیک ترمینال</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>پایان موفق job، خروجی آماده</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>روی فریم ظاهرشدن خروجی</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>−۱۲ dB</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>1.00s</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>prompt_tick</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>تیک ظهور prompt</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>آمدن خط prompt جدید</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>روی فریم ظهور $ یا #</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>−۱۶ dB</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>0.05s</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>تایپ و ترمینال</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>scroll_ratchet</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>اسکرول رچتی</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>اسکرول لاگ، man page</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>هم‌زمان با حرکت اسکرول</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>−۱۴ dB</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>0.50s</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>فضاسازی (لوپ)</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>room_tone_loop</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>نویز اتاق + هوم + فن</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>زیر کل ویدیو برای پرکردن سکوت مطلق</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Loop از ابتدا تا انتها، بدون قطع</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>−۳۴ تا −۳۰ dB</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>30.00s</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>فضاسازی (لوپ)</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>vinyl_crackle_loop</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>کرکل صفحه‌ی گرامافون</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>حال‌وهوای لوفای/نوستالژیک، زیر موزیک آرام</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Loop؛ حجم خیلی کم</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>−۲۴ dB</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>9.00s</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G32"/>
+  <autoFilter ref="A1:G41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1679,7 +2012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2017,45 +2350,85 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>bgm_terminal_flow</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>مینیمال تاریک-خنثی: پالس ساب + پلاک پنتاتونیک + اکو</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>کدنویسی زنده، تیم‌لپس تایپ، جلسه‌های ترمینال لینوکس</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>36.5s</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Am – F – C – G (واز باز)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>بله</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>−۲۲ dB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>bgm_cinematic_tension</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B10" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>تیره و پرتنش با ریزر و ضربه‌ی پایانی</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>مقایسه‌ی حساس، تست دوام، «مشکل اینجاست»</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>30.0s</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Am – F – Gm – Em</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>بله</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>−۲۰ dB</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2644,7 +3017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2927,103 +3300,103 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>ریلز / شورتس</t>
+          <t>آموزش کد / لینوکس</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>0.0–0.5</t>
+          <t>تایپ دیده‌شده</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ضربه‌ی اول</t>
+          <t>B-roll تایپ</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>impact_deep یا boom_cinematic</t>
+          <t>type_burst_mech همگام + bgm_terminal_flow</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>بدون استثنا؛ قوی‌ترین افکت پک</t>
+          <t>Rate Stretch با سرعت واقعی</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ریلز / شورتس</t>
+          <t>آموزش کد / لینوکس</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>0.5–3</t>
+          <t>تایپ زیر نریشن</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>بستر</t>
+          <t>نریشن هم‌زمان</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>bgm_hook_loop_8s روی لوپ + cut_tick روی هر کات</t>
+          <t>type_burst_soft @ −۱۸ dB</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ریتم تند</t>
+          <t>هرگز نوع مکانیکی زیر نریشن نه</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>ریلز / شورتس</t>
+          <t>آموزش کد / لینوکس</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>هر متن</t>
+          <t>اجرای دستور</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>ظهور متن</t>
+          <t>فریم Enter</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>text_reveal_soft یا pop_bubble</t>
+          <t>type_enter + prompt_tick</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>prompt_tick بعد از ظهور خروجی</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ریلز / شورتس</t>
+          <t>آموزش کد / لینوکس</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>لحظه‌ی «واو»</t>
+          <t>خطا / موفقیت</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>اوج</t>
+          <t>خروجی قرمز / سبز</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>sparkle_magic یا success_chime</t>
+          <t>error_buzz یا terminal_bell + success_chime</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3040,22 +3413,22 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>شوخی</t>
+          <t>0.0–0.5</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>میم</t>
+          <t>ضربه‌ی اول</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>air_horn_meme یا laser_pew</t>
+          <t>impact_deep یا boom_cinematic</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>بدون استثنا؛ قوی‌ترین افکت پک</t>
         </is>
       </c>
     </row>
@@ -3067,81 +3440,189 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>پایان/CTA</t>
+          <t>0.5–3</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>خاتمه</t>
+          <t>بستر</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>vinyl_stop + logo_sting کوتاه</t>
+          <t>bgm_hook_loop_8s روی لوپ + cut_tick روی هر کات</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ریتم تند</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>استوری/پست اینستاگرام</t>
+          <t>ریلز / شورتس</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>0–1</t>
+          <t>هر متن</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>قلاب</t>
+          <t>ظهور متن</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>impact_bright + zoom-in تصویری</t>
+          <t>text_reveal_soft یا pop_bubble</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>صدا در اینستاگرام خودکار پخش می‌شود؛ ۱ ثانیه‌ی اول حیاتی است</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>ریلز / شورتس</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>لحظه‌ی «واو»</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>اوج</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>sparkle_magic یا success_chime</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ریلز / شورتس</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>شوخی</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>میم</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>air_horn_meme یا laser_pew</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ریلز / شورتس</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>پایان/CTA</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>خاتمه</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>vinyl_stop + logo_sting کوتاه</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>استوری/پست اینستاگرام</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>قلاب</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>impact_bright + zoom-in تصویری</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>صدا در اینستاگرام خودکار پخش می‌شود؛ ۱ ثانیه‌ی اول حیاتی است</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>استوری/پست اینستاگرام</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>ریتم</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>cut_tick روی هر کات + bgm_screen_bed</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>اگر موزیک ترند اینستاگرام را می‌گذاری، حجمش را −۲۴ dB کن و افکت خودت را رویش بچین</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E18"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>